<commit_message>
feat: clean up legacy code and implement project details tabbed sidebar layout
</commit_message>
<xml_diff>
--- a/Data/DSP Material Expense.xlsx
+++ b/Data/DSP Material Expense.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d772b42a7a1256b2/Desktop/Business/TSK Constructions/Projects/Building Construction/DSP Site Podanur/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="399" documentId="13_ncr:1_{81555393-077D-47DF-B99E-C2CBB59417EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E07EC3ED-03DD-4B59-B393-EF5CB43CE046}"/>
+  <xr:revisionPtr revIDLastSave="501" documentId="13_ncr:1_{81555393-077D-47DF-B99E-C2CBB59417EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03E27704-7A41-4AF2-A1D9-9FDF6AEB2C81}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="60">
   <si>
     <t>DATE</t>
   </si>
@@ -226,6 +226,24 @@
   </si>
   <si>
     <t>Brick Paymen 5000 nos</t>
+  </si>
+  <si>
+    <t>Pending amt</t>
+  </si>
+  <si>
+    <t>RAMDEV HARDWARES</t>
+  </si>
+  <si>
+    <t>23-05026</t>
+  </si>
+  <si>
+    <t>CHQ</t>
+  </si>
+  <si>
+    <t>CHQ from School Site</t>
+  </si>
+  <si>
+    <t>Part Payment-CHQ from School</t>
   </si>
 </sst>
 </file>
@@ -397,7 +415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -430,6 +448,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1717,100 +1737,179 @@
       <c r="I28" s="6"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A29" s="10"/>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="19"/>
+      <c r="A29" s="10">
+        <v>46156</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="E29" s="18">
+        <v>100</v>
+      </c>
+      <c r="F29" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="G29" s="19">
+        <v>295</v>
+      </c>
       <c r="H29" s="11">
         <f>Table1[[#This Row],[QTY]]*Table1[[#This Row],[RATE]]</f>
-        <v>0</v>
+        <v>29500</v>
       </c>
       <c r="I29" s="6"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A30" s="17"/>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
+      <c r="A30" s="17">
+        <v>46157</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" s="18">
+        <v>2721</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>13</v>
+      </c>
       <c r="G30" s="19"/>
       <c r="H30" s="20">
-        <f>Table1[[#This Row],[QTY]]*Table1[[#This Row],[RATE]]</f>
-        <v>0</v>
+        <v>209880</v>
       </c>
       <c r="I30" s="6"/>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A31" s="10"/>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
+      <c r="A31" s="10">
+        <v>46162</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E31" s="6">
+        <v>892</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>13</v>
+      </c>
       <c r="G31" s="7"/>
       <c r="H31" s="20">
-        <f>Table1[[#This Row],[QTY]]*Table1[[#This Row],[RATE]]</f>
-        <v>0</v>
+        <v>70380</v>
       </c>
       <c r="I31" s="6"/>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A32" s="17"/>
-      <c r="B32" s="18"/>
+      <c r="A32" s="17">
+        <v>46165</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>18</v>
+      </c>
       <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="19"/>
+      <c r="D32" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E32" s="18">
+        <v>8</v>
+      </c>
+      <c r="F32" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G32" s="19">
+        <v>4700</v>
+      </c>
       <c r="H32" s="20">
         <f>Table1[[#This Row],[QTY]]*Table1[[#This Row],[RATE]]</f>
-        <v>0</v>
+        <v>37600</v>
       </c>
       <c r="I32" s="6"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A33" s="17"/>
-      <c r="B33" s="18"/>
+      <c r="A33" s="17">
+        <v>46165</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>20</v>
+      </c>
       <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="19"/>
+      <c r="D33" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E33" s="18">
+        <v>8</v>
+      </c>
+      <c r="F33" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G33" s="19">
+        <v>4125</v>
+      </c>
       <c r="H33" s="20">
         <f>Table1[[#This Row],[QTY]]*Table1[[#This Row],[RATE]]</f>
-        <v>0</v>
+        <v>33000</v>
       </c>
       <c r="I33" s="6"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" s="17"/>
-      <c r="B34" s="18"/>
+      <c r="A34" s="17">
+        <v>46165</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>29</v>
+      </c>
       <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
+      <c r="D34" s="18" t="s">
+        <v>55</v>
+      </c>
       <c r="E34" s="18"/>
       <c r="F34" s="18"/>
       <c r="G34" s="19"/>
       <c r="H34" s="20">
-        <f>Table1[[#This Row],[QTY]]*Table1[[#This Row],[RATE]]</f>
-        <v>0</v>
+        <v>9211</v>
       </c>
       <c r="I34" s="6"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A35" s="10"/>
-      <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="7"/>
+      <c r="A35" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E35" s="6">
+        <v>50</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G35" s="7">
+        <v>295</v>
+      </c>
       <c r="H35" s="11">
         <f>Table1[[#This Row],[QTY]]*Table1[[#This Row],[RATE]]</f>
-        <v>0</v>
+        <v>14750</v>
       </c>
       <c r="I35" s="6"/>
     </row>
@@ -1980,7 +2079,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DC52B97-F8EC-489B-AAAD-008E3D44EA2D}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -2004,19 +2103,19 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="str" cm="1">
-        <f t="array" ref="A2:A10">_xlfn.UNIQUE('Material Details'!B2:B1008)</f>
+        <f t="array" ref="A2:A11">_xlfn.UNIQUE('Material Details'!B2:B1008)</f>
         <v>CEMENT</v>
       </c>
       <c r="B2" s="6">
         <f>SUMIF('Material Details'!B2:B1008,A2,'Material Details'!E2:E1008)</f>
-        <v>470</v>
+        <v>620</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D2" s="7">
         <f>SUMIF('Material Details'!B2:B1008,A2,'Material Details'!H2:H1008)</f>
-        <v>130900</v>
+        <v>175150</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -2025,14 +2124,14 @@
       </c>
       <c r="B3" s="6">
         <f>SUMIF('Material Details'!B3:B1009,A3,'Material Details'!E3:E1009)</f>
-        <v>4827</v>
+        <v>8440</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="7">
         <f>SUMIF('Material Details'!B3:B1009,A3,'Material Details'!H3:H1009)</f>
-        <v>379580</v>
+        <v>659840</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -2041,14 +2140,14 @@
       </c>
       <c r="B4" s="6">
         <f>SUMIF('Material Details'!B4:B1010,A4,'Material Details'!E4:E1010)</f>
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="7">
         <f>SUMIF('Material Details'!B4:B1010,A4,'Material Details'!H4:H1010)</f>
-        <v>112800</v>
+        <v>150400</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -2057,14 +2156,14 @@
       </c>
       <c r="B5" s="6">
         <f>SUMIF('Material Details'!B5:B1011,A5,'Material Details'!E5:E1011)</f>
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>17</v>
       </c>
       <c r="D5" s="7">
         <f>SUMIF('Material Details'!B5:B1011,A5,'Material Details'!H5:H1011)</f>
-        <v>49500</v>
+        <v>82500</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -2132,7 +2231,12 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10">
+      <c r="A10" t="str">
+        <v>ELECTRICAL</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11">
         <v>0</v>
       </c>
     </row>
@@ -2143,7 +2247,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D96697B0-05D6-4BCA-A61B-0D246D1FF2DE}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.54296875" bestFit="1" customWidth="1"/>
@@ -2168,7 +2272,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="str" cm="1">
-        <f t="array" ref="A2:A10">_xlfn.UNIQUE('Material Details'!D2:D1008)</f>
+        <f t="array" ref="A2:A11">_xlfn.UNIQUE('Material Details'!D2:D1008)</f>
         <v>NV ASSOCIATES</v>
       </c>
       <c r="B2" s="7">
@@ -2211,11 +2315,11 @@
       </c>
       <c r="C4" s="7">
         <f>SUMIF('Payment Details'!B2:B991,'Vendor Balance Sheet'!A4,'Payment Details'!C2:C991)</f>
-        <v>80000</v>
+        <v>88400</v>
       </c>
       <c r="D4" s="7">
         <f t="shared" si="0"/>
-        <v>8400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -2224,15 +2328,15 @@
       </c>
       <c r="B5" s="7">
         <f>SUMIF('Material Details'!D4:D1010,A5,'Material Details'!H4:H1010)</f>
-        <v>190300</v>
+        <v>260900</v>
       </c>
       <c r="C5" s="7">
         <f>SUMIF('Payment Details'!B2:B992,'Vendor Balance Sheet'!A5,'Payment Details'!C2:C992)</f>
-        <v>150000</v>
+        <v>225000</v>
       </c>
       <c r="D5" s="7">
         <f t="shared" si="0"/>
-        <v>40300</v>
+        <v>35900</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -2258,15 +2362,15 @@
       </c>
       <c r="B7" s="7">
         <f>SUMIF('Material Details'!D6:D1012,A7,'Material Details'!H6:H1012)</f>
-        <v>230180</v>
+        <v>510440</v>
       </c>
       <c r="C7" s="7">
         <f>SUMIF('Payment Details'!B4:B994,'Vendor Balance Sheet'!A7,'Payment Details'!C4:C994)</f>
-        <v>200000</v>
+        <v>500000</v>
       </c>
       <c r="D7" s="7">
         <f t="shared" si="0"/>
-        <v>30180</v>
+        <v>10440</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -2275,15 +2379,15 @@
       </c>
       <c r="B8" s="7">
         <f>SUMIF('Material Details'!D7:D1013,A8,'Material Details'!H7:H1013)</f>
-        <v>28750</v>
+        <v>73000</v>
       </c>
       <c r="C8" s="7">
         <f>SUMIF('Payment Details'!B5:B995,'Vendor Balance Sheet'!A8,'Payment Details'!C5:C995)</f>
-        <v>13500</v>
+        <v>49000</v>
       </c>
       <c r="D8" s="7">
         <f t="shared" ref="D8" si="1">B8-C8</f>
-        <v>15250</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -2304,7 +2408,24 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10">
+      <c r="A10" s="6" t="str">
+        <v>RAMDEV HARDWARES</v>
+      </c>
+      <c r="B10" s="7">
+        <f>SUMIF('Material Details'!D9:D1015,A10,'Material Details'!H9:H1015)</f>
+        <v>9211</v>
+      </c>
+      <c r="C10" s="7">
+        <f>SUMIF('Payment Details'!B7:B997,'Vendor Balance Sheet'!A10,'Payment Details'!C7:C997)</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="7">
+        <f t="shared" ref="D10" si="3">B10-C10</f>
+        <v>9211</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11">
         <v>0</v>
       </c>
     </row>
@@ -2315,7 +2436,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B843CC5F-739E-45E9-AC65-8442CF552E38}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="3"/>
@@ -2667,52 +2788,144 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="5"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="A18" s="5">
+        <v>46158</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="7">
+        <v>25000</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="5"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
+      <c r="A19" s="5">
+        <v>46158</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="7">
+        <v>8400</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" s="5"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
+      <c r="A20" s="5">
+        <v>46158</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" s="7">
+        <v>30000</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
+      <c r="A21" s="5">
+        <v>46172</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C21" s="7">
+        <v>50000</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" s="5"/>
-      <c r="B22" s="6"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
+      <c r="A22" s="5">
+        <v>46172</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="7">
+        <v>200000</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="5"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
+      <c r="A23" s="5">
+        <v>46179</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" s="7">
+        <v>100000</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="3">
+        <v>46179</v>
+      </c>
+      <c r="B24" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="C24" s="4">
+        <v>5500</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F24" s="25" t="s">
+        <v>46</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1" xr:uid="{B843CC5F-739E-45E9-AC65-8442CF552E38}"/>

</xml_diff>